<commit_message>
CFG + path coverage + loop coverage
</commit_message>
<xml_diff>
--- a/docs/Lab02/Lab02_BBT__TCs_Form.xlsx
+++ b/docs/Lab02/Lab02_BBT__TCs_Form.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cezar1000000\IdeaProjects\vvss\docs\Lab02\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B63EB45-4D7C-4C75-86B7-5A19D259B27F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25180242-D057-4932-89BD-5E9B3FCB1C5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{A8EE5D2A-0D12-42FF-81F5-0F6BE23884CE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A8EE5D2A-0D12-42FF-81F5-0F6BE23884CE}"/>
   </bookViews>
   <sheets>
     <sheet name="Statement" sheetId="4" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="95">
   <si>
     <t>VVSS, Info Romana, 2025-2026</t>
   </si>
@@ -238,9 +238,6 @@
     <t>Gaspar Dan</t>
   </si>
   <si>
-    <t>1. Adaugarea unui produs</t>
-  </si>
-  <si>
     <t>F01. adaugarea unui produs nou (nume, pret, categorie, tip)</t>
   </si>
   <si>
@@ -269,9 +266,6 @@
   </si>
   <si>
     <t>TC1_ECP</t>
-  </si>
-  <si>
-    <t>-</t>
   </si>
   <si>
     <t>…</t>
@@ -362,6 +356,9 @@
   </si>
   <si>
     <t>TC6_BVA</t>
+  </si>
+  <si>
+    <t>1. Gestionarea produselor</t>
   </si>
 </sst>
 </file>
@@ -919,7 +916,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="111">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -957,81 +954,7 @@
     <xf numFmtId="2" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1043,21 +966,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1101,6 +1009,106 @@
     <xf numFmtId="0" fontId="17" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1119,7 +1127,34 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1137,56 +1172,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1530,18 +1524,18 @@
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
-      <c r="C1" s="61" t="s">
+      <c r="C1" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="50" t="s">
+      <c r="H1" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="I1" s="50"/>
-      <c r="J1" s="50"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
@@ -1556,11 +1550,11 @@
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="57" t="s">
+      <c r="H2" s="53" t="s">
         <v>49</v>
       </c>
-      <c r="I2" s="58"/>
-      <c r="J2" s="59"/>
+      <c r="I2" s="54"/>
+      <c r="J2" s="55"/>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
@@ -1636,7 +1630,7 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
-      <c r="B6" s="52"/>
+      <c r="B6" s="26"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -1676,7 +1670,7 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
-      <c r="B8" s="53" t="s">
+      <c r="B8" s="27" t="s">
         <v>55</v>
       </c>
       <c r="C8" s="1"/>
@@ -1787,7 +1781,7 @@
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="1" t="s">
-        <v>62</v>
+        <v>94</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
@@ -1806,7 +1800,7 @@
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
@@ -1825,7 +1819,7 @@
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
@@ -1860,7 +1854,7 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
-      <c r="B18" s="53"/>
+      <c r="B18" s="27"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
@@ -1895,7 +1889,7 @@
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
-      <c r="C20" s="54"/>
+      <c r="C20" s="28"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
@@ -1961,20 +1955,20 @@
       <c r="O23" s="5"/>
     </row>
     <row r="24" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="55"/>
-      <c r="B24" s="60"/>
-      <c r="C24" s="60"/>
-      <c r="D24" s="60"/>
-      <c r="E24" s="60"/>
-      <c r="F24" s="60"/>
-      <c r="G24" s="60"/>
-      <c r="H24" s="60"/>
-      <c r="I24" s="60"/>
-      <c r="J24" s="60"/>
-      <c r="K24" s="60"/>
-      <c r="L24" s="60"/>
-      <c r="M24" s="60"/>
-      <c r="N24" s="60"/>
+      <c r="A24" s="29"/>
+      <c r="B24" s="56"/>
+      <c r="C24" s="56"/>
+      <c r="D24" s="56"/>
+      <c r="E24" s="56"/>
+      <c r="F24" s="56"/>
+      <c r="G24" s="56"/>
+      <c r="H24" s="56"/>
+      <c r="I24" s="56"/>
+      <c r="J24" s="56"/>
+      <c r="K24" s="56"/>
+      <c r="L24" s="56"/>
+      <c r="M24" s="56"/>
+      <c r="N24" s="56"/>
       <c r="O24" s="1"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
@@ -1997,7 +1991,7 @@
     <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
-      <c r="C26" s="56"/>
+      <c r="C26" s="30"/>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
@@ -2035,14 +2029,14 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
-      <c r="B1" s="37" t="s">
+      <c r="B1" s="71" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
@@ -2060,8 +2054,8 @@
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
@@ -2075,12 +2069,12 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="59" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
       <c r="H3" s="1"/>
@@ -2100,8 +2094,8 @@
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
+      <c r="F4" s="57"/>
+      <c r="G4" s="57"/>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
@@ -2115,22 +2109,22 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
-      <c r="B5" s="39" t="s">
+      <c r="B5" s="73" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="40"/>
-      <c r="D5" s="40"/>
-      <c r="E5" s="41"/>
+      <c r="C5" s="74"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="1"/>
-      <c r="G5" s="28" t="s">
+      <c r="G5" s="62" t="s">
         <v>2</v>
       </c>
-      <c r="H5" s="29"/>
-      <c r="I5" s="29"/>
-      <c r="J5" s="29"/>
-      <c r="K5" s="29"/>
-      <c r="L5" s="29"/>
-      <c r="M5" s="29"/>
+      <c r="H5" s="63"/>
+      <c r="I5" s="63"/>
+      <c r="J5" s="63"/>
+      <c r="K5" s="63"/>
+      <c r="L5" s="63"/>
+      <c r="M5" s="63"/>
       <c r="N5" s="10"/>
       <c r="O5" s="5"/>
       <c r="P5" s="5"/>
@@ -2151,18 +2145,18 @@
         <v>6</v>
       </c>
       <c r="F6" s="1"/>
-      <c r="G6" s="33" t="s">
+      <c r="G6" s="67" t="s">
         <v>7</v>
       </c>
-      <c r="H6" s="35" t="s">
+      <c r="H6" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="I6" s="26" t="s">
+      <c r="I6" s="60" t="s">
         <v>9</v>
       </c>
-      <c r="J6" s="27"/>
-      <c r="K6" s="27"/>
-      <c r="L6" s="27"/>
+      <c r="J6" s="61"/>
+      <c r="K6" s="61"/>
+      <c r="L6" s="61"/>
       <c r="M6" s="9" t="s">
         <v>10</v>
       </c>
@@ -2173,7 +2167,7 @@
       <c r="B7" s="3">
         <v>1</v>
       </c>
-      <c r="C7" s="31" t="s">
+      <c r="C7" s="65" t="s">
         <v>13</v>
       </c>
       <c r="D7" s="3" t="s">
@@ -2181,8 +2175,8 @@
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="1"/>
-      <c r="G7" s="34"/>
-      <c r="H7" s="36"/>
+      <c r="G7" s="68"/>
+      <c r="H7" s="70"/>
       <c r="I7" s="2" t="s">
         <v>20</v>
       </c>
@@ -2205,7 +2199,7 @@
       <c r="B8" s="3">
         <v>2</v>
       </c>
-      <c r="C8" s="32"/>
+      <c r="C8" s="66"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
         <v>16</v>
@@ -2239,7 +2233,7 @@
       <c r="B9" s="3">
         <v>3</v>
       </c>
-      <c r="C9" s="31" t="s">
+      <c r="C9" s="65" t="s">
         <v>17</v>
       </c>
       <c r="D9" s="3" t="s">
@@ -2275,7 +2269,7 @@
       <c r="B10" s="3">
         <v>4</v>
       </c>
-      <c r="C10" s="32"/>
+      <c r="C10" s="66"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3" t="s">
         <v>19</v>
@@ -2307,7 +2301,7 @@
     <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="6"/>
-      <c r="C11" s="30"/>
+      <c r="C11" s="64"/>
       <c r="D11" s="6"/>
       <c r="E11" s="6"/>
       <c r="F11" s="1"/>
@@ -2316,7 +2310,7 @@
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="6"/>
-      <c r="C12" s="30"/>
+      <c r="C12" s="64"/>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
       <c r="F12" s="1"/>
@@ -2325,7 +2319,7 @@
     <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="6"/>
-      <c r="C13" s="30"/>
+      <c r="C13" s="64"/>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
       <c r="F13" s="1"/>
@@ -2334,7 +2328,7 @@
     <row r="14" spans="1:17" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="6"/>
-      <c r="C14" s="30"/>
+      <c r="C14" s="64"/>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
       <c r="F14" s="1"/>
@@ -2343,7 +2337,7 @@
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="6"/>
-      <c r="C15" s="30"/>
+      <c r="C15" s="64"/>
       <c r="D15" s="6"/>
       <c r="E15" s="6"/>
       <c r="F15" s="1"/>
@@ -2352,7 +2346,7 @@
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="6"/>
-      <c r="C16" s="30"/>
+      <c r="C16" s="64"/>
       <c r="D16" s="6"/>
       <c r="E16" s="6"/>
       <c r="F16" s="1"/>
@@ -2361,7 +2355,7 @@
     <row r="17" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="6"/>
-      <c r="C17" s="30"/>
+      <c r="C17" s="64"/>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
       <c r="F17" s="1"/>
@@ -2380,7 +2374,7 @@
     <row r="18" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="6"/>
-      <c r="C18" s="30"/>
+      <c r="C18" s="64"/>
       <c r="D18" s="6"/>
       <c r="E18" s="6"/>
       <c r="F18" s="1"/>
@@ -2399,7 +2393,7 @@
     <row r="19" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="6"/>
-      <c r="C19" s="30"/>
+      <c r="C19" s="64"/>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
       <c r="F19" s="1"/>
@@ -2418,11 +2412,11 @@
     <row r="20" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="6"/>
-      <c r="C20" s="30"/>
+      <c r="C20" s="64"/>
       <c r="D20" s="6"/>
       <c r="E20" s="6"/>
-      <c r="F20" s="23"/>
-      <c r="G20" s="23"/>
+      <c r="F20" s="57"/>
+      <c r="G20" s="57"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
@@ -2440,8 +2434,8 @@
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
-      <c r="F21" s="23"/>
-      <c r="G21" s="23"/>
+      <c r="F21" s="57"/>
+      <c r="G21" s="57"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
@@ -2461,8 +2455,8 @@
         <v>12</v>
       </c>
       <c r="E22" s="1"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="24"/>
+      <c r="F22" s="58"/>
+      <c r="G22" s="58"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
@@ -2520,103 +2514,103 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B1" s="37" t="s">
+      <c r="B1" s="71" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
     </row>
     <row r="3" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B3" s="25" t="s">
-        <v>91</v>
-      </c>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="105"/>
-      <c r="F3" s="107"/>
-      <c r="G3" s="106"/>
+      <c r="B3" s="59" t="s">
+        <v>89</v>
+      </c>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="77"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="5"/>
     </row>
     <row r="5" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B5" s="42" t="s">
+      <c r="B5" s="80" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="43"/>
-      <c r="D5" s="44"/>
+      <c r="C5" s="81"/>
+      <c r="D5" s="82"/>
     </row>
     <row r="6" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B6" s="45" t="s">
+      <c r="B6" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="45" t="s">
+      <c r="C6" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="45" t="s">
+      <c r="D6" s="23" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="2:19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="46">
+      <c r="B7" s="76">
         <v>1</v>
       </c>
-      <c r="C7" s="46" t="s">
+      <c r="C7" s="76" t="s">
         <v>38</v>
       </c>
-      <c r="D7" s="45" t="s">
+      <c r="D7" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="K7" s="46" t="s">
+      <c r="K7" s="76" t="s">
         <v>40</v>
       </c>
-      <c r="L7" s="46" t="s">
+      <c r="L7" s="76" t="s">
         <v>41</v>
       </c>
-      <c r="M7" s="48" t="s">
+      <c r="M7" s="78" t="s">
         <v>46</v>
       </c>
-      <c r="N7" s="48" t="s">
+      <c r="N7" s="78" t="s">
         <v>47</v>
       </c>
-      <c r="O7" s="46" t="s">
+      <c r="O7" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="P7" s="46"/>
-      <c r="Q7" s="46"/>
-      <c r="R7" s="46"/>
-      <c r="S7" s="45" t="s">
+      <c r="P7" s="76"/>
+      <c r="Q7" s="76"/>
+      <c r="R7" s="76"/>
+      <c r="S7" s="23" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="8" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B8" s="46"/>
-      <c r="C8" s="46"/>
-      <c r="D8" s="45" t="s">
+      <c r="B8" s="76"/>
+      <c r="C8" s="76"/>
+      <c r="D8" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="K8" s="46"/>
-      <c r="L8" s="46"/>
-      <c r="M8" s="49"/>
-      <c r="N8" s="49"/>
-      <c r="O8" s="45" t="s">
+      <c r="K8" s="76"/>
+      <c r="L8" s="76"/>
+      <c r="M8" s="79"/>
+      <c r="N8" s="79"/>
+      <c r="O8" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="P8" s="45" t="s">
+      <c r="P8" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="Q8" s="45" t="s">
+      <c r="Q8" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="R8" s="45" t="s">
+      <c r="R8" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="S8" s="45" t="s">
+      <c r="S8" s="23" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="9" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B9" s="46"/>
-      <c r="C9" s="46"/>
-      <c r="D9" s="45" t="s">
+      <c r="B9" s="76"/>
+      <c r="C9" s="76"/>
+      <c r="D9" s="23" t="s">
         <v>37</v>
       </c>
       <c r="K9" s="2">
@@ -2644,13 +2638,13 @@
       </c>
     </row>
     <row r="10" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B10" s="46">
+      <c r="B10" s="76">
         <v>2</v>
       </c>
-      <c r="C10" s="46" t="s">
+      <c r="C10" s="76" t="s">
         <v>39</v>
       </c>
-      <c r="D10" s="47" t="s">
+      <c r="D10" s="23" t="s">
         <v>42</v>
       </c>
       <c r="K10" s="2">
@@ -2678,9 +2672,9 @@
       </c>
     </row>
     <row r="11" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B11" s="46"/>
-      <c r="C11" s="46"/>
-      <c r="D11" s="47" t="s">
+      <c r="B11" s="76"/>
+      <c r="C11" s="76"/>
+      <c r="D11" s="23" t="s">
         <v>43</v>
       </c>
       <c r="K11" s="2">
@@ -2708,9 +2702,9 @@
       </c>
     </row>
     <row r="12" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B12" s="46"/>
-      <c r="C12" s="46"/>
-      <c r="D12" s="47" t="s">
+      <c r="B12" s="76"/>
+      <c r="C12" s="76"/>
+      <c r="D12" s="23" t="s">
         <v>44</v>
       </c>
       <c r="K12" s="2">
@@ -2789,9 +2783,6 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="K7:K8"/>
     <mergeCell ref="L7:L8"/>
     <mergeCell ref="O7:R7"/>
     <mergeCell ref="M7:M8"/>
@@ -2801,6 +2792,9 @@
     <mergeCell ref="C7:C9"/>
     <mergeCell ref="B10:B12"/>
     <mergeCell ref="C10:C12"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="K7:K8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2817,12 +2811,12 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
-      <c r="B1" s="37" t="s">
+      <c r="B1" s="71" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
@@ -2855,89 +2849,87 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
-      <c r="B3" s="108" t="s">
-        <v>65</v>
-      </c>
-      <c r="C3" s="109"/>
-      <c r="D3" s="109"/>
-      <c r="E3" s="109"/>
-      <c r="F3" s="109"/>
-      <c r="G3" s="109"/>
-      <c r="H3" s="109"/>
-      <c r="I3" s="109"/>
-      <c r="J3" s="109"/>
-      <c r="K3" s="110"/>
+      <c r="B3" s="49" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" s="50"/>
+      <c r="D3" s="50"/>
+      <c r="E3" s="50"/>
+      <c r="F3" s="50"/>
+      <c r="G3" s="50"/>
+      <c r="H3" s="50"/>
+      <c r="I3" s="50"/>
+      <c r="J3" s="50"/>
+      <c r="K3" s="51"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
-      <c r="B4" s="33" t="s">
+      <c r="B4" s="67" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" s="85" t="s">
         <v>66</v>
       </c>
-      <c r="C4" s="80" t="s">
+      <c r="D4" s="87" t="s">
         <v>67</v>
       </c>
-      <c r="D4" s="82" t="s">
+      <c r="E4" s="69" t="s">
         <v>68</v>
       </c>
-      <c r="E4" s="35" t="s">
-        <v>69</v>
-      </c>
-      <c r="F4" s="46" t="s">
+      <c r="F4" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="46"/>
-      <c r="H4" s="46"/>
-      <c r="I4" s="46"/>
-      <c r="J4" s="26" t="s">
+      <c r="G4" s="76"/>
+      <c r="H4" s="76"/>
+      <c r="I4" s="76"/>
+      <c r="J4" s="60" t="s">
         <v>10</v>
       </c>
-      <c r="K4" s="85"/>
+      <c r="K4" s="83"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
     </row>
     <row r="5" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1"/>
-      <c r="B5" s="79"/>
-      <c r="C5" s="81"/>
-      <c r="D5" s="83"/>
-      <c r="E5" s="84"/>
-      <c r="F5" s="45" t="s">
+      <c r="B5" s="84"/>
+      <c r="C5" s="86"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="89"/>
+      <c r="F5" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="45" t="s">
+      <c r="G5" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="H5" s="45" t="s">
+      <c r="H5" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="45" t="s">
+      <c r="I5" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="J5" s="63" t="s">
+      <c r="J5" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="K5" s="63" t="s">
-        <v>70</v>
+      <c r="K5" s="32" t="s">
+        <v>69</v>
       </c>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
     </row>
     <row r="6" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
-      <c r="B6" s="64">
+      <c r="B6" s="33">
         <v>1</v>
       </c>
-      <c r="C6" s="104" t="s">
+      <c r="C6" s="107" t="s">
+        <v>70</v>
+      </c>
+      <c r="D6" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="D6" s="65" t="s">
-        <v>72</v>
-      </c>
-      <c r="E6" s="64" t="s">
-        <v>73</v>
-      </c>
+      <c r="E6" s="33"/>
       <c r="F6" s="4" t="s">
         <v>24</v>
       </c>
@@ -2953,24 +2945,22 @@
       <c r="J6" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="K6" s="64" t="s">
-        <v>74</v>
+      <c r="K6" s="33" t="s">
+        <v>72</v>
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
-      <c r="B7" s="66">
+      <c r="B7" s="35">
         <v>2</v>
       </c>
-      <c r="C7" s="104"/>
-      <c r="D7" s="67" t="s">
-        <v>92</v>
-      </c>
-      <c r="E7" s="66" t="s">
-        <v>73</v>
-      </c>
+      <c r="C7" s="107"/>
+      <c r="D7" s="36" t="s">
+        <v>90</v>
+      </c>
+      <c r="E7" s="35"/>
       <c r="F7" s="18" t="s">
         <v>28</v>
       </c>
@@ -2986,24 +2976,22 @@
       <c r="J7" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="K7" s="66" t="s">
-        <v>74</v>
+      <c r="K7" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
-      <c r="B8" s="66">
+      <c r="B8" s="35">
         <v>3</v>
       </c>
-      <c r="C8" s="104"/>
-      <c r="D8" s="67" t="s">
-        <v>75</v>
-      </c>
-      <c r="E8" s="66" t="s">
+      <c r="C8" s="107"/>
+      <c r="D8" s="36" t="s">
         <v>73</v>
       </c>
+      <c r="E8" s="35"/>
       <c r="F8" s="17" t="s">
         <v>24</v>
       </c>
@@ -3019,23 +3007,21 @@
       <c r="J8" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="K8" s="66" t="s">
-        <v>74</v>
+      <c r="K8" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
-      <c r="B9" s="66">
+      <c r="B9" s="35">
         <v>4</v>
       </c>
-      <c r="C9" s="104"/>
-      <c r="D9" s="67" t="s">
-        <v>74</v>
-      </c>
-      <c r="E9" s="66" t="s">
-        <v>93</v>
+      <c r="C9" s="107"/>
+      <c r="D9" s="36"/>
+      <c r="E9" s="35" t="s">
+        <v>91</v>
       </c>
       <c r="F9" s="17" t="s">
         <v>24</v>
@@ -3052,23 +3038,21 @@
       <c r="J9" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="K9" s="66" t="s">
-        <v>74</v>
+      <c r="K9" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
-      <c r="B10" s="66">
+      <c r="B10" s="35">
         <v>5</v>
       </c>
-      <c r="C10" s="104"/>
-      <c r="D10" s="67" t="s">
-        <v>73</v>
-      </c>
-      <c r="E10" s="66" t="s">
-        <v>94</v>
+      <c r="C10" s="107"/>
+      <c r="D10" s="36"/>
+      <c r="E10" s="35" t="s">
+        <v>92</v>
       </c>
       <c r="F10" s="18" t="s">
         <v>30</v>
@@ -3085,23 +3069,21 @@
       <c r="J10" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="K10" s="66" t="s">
-        <v>74</v>
+      <c r="K10" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
-      <c r="B11" s="66">
+      <c r="B11" s="35">
         <v>6</v>
       </c>
-      <c r="C11" s="104"/>
-      <c r="D11" s="67" t="s">
-        <v>73</v>
-      </c>
-      <c r="E11" s="66" t="s">
-        <v>76</v>
+      <c r="C11" s="107"/>
+      <c r="D11" s="36"/>
+      <c r="E11" s="35" t="s">
+        <v>74</v>
       </c>
       <c r="F11" s="18" t="s">
         <v>31</v>
@@ -3118,23 +3100,21 @@
       <c r="J11" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="K11" s="66" t="s">
-        <v>74</v>
+      <c r="K11" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
-      <c r="B12" s="66">
+      <c r="B12" s="35">
         <v>7</v>
       </c>
-      <c r="C12" s="104"/>
-      <c r="D12" s="67" t="s">
-        <v>73</v>
-      </c>
-      <c r="E12" s="66" t="s">
-        <v>77</v>
+      <c r="C12" s="107"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="35" t="s">
+        <v>75</v>
       </c>
       <c r="F12" s="17" t="s">
         <v>24</v>
@@ -3151,21 +3131,21 @@
       <c r="J12" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="K12" s="66" t="s">
-        <v>74</v>
+      <c r="K12" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
-      <c r="B13" s="103">
+      <c r="B13" s="48">
         <v>8</v>
       </c>
-      <c r="C13" s="104"/>
-      <c r="D13" s="62"/>
-      <c r="E13" s="103" t="s">
-        <v>78</v>
+      <c r="C13" s="107"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="48" t="s">
+        <v>76</v>
       </c>
       <c r="F13" s="17" t="s">
         <v>24</v>
@@ -3182,21 +3162,21 @@
       <c r="J13" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="K13" s="103"/>
+      <c r="K13" s="48" t="s">
+        <v>72</v>
+      </c>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
     </row>
     <row r="14" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1"/>
-      <c r="B14" s="69">
+      <c r="B14" s="38">
         <v>9</v>
       </c>
-      <c r="C14" s="104"/>
-      <c r="D14" s="70" t="s">
-        <v>74</v>
-      </c>
-      <c r="E14" s="69" t="s">
-        <v>95</v>
+      <c r="C14" s="107"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="38" t="s">
+        <v>93</v>
       </c>
       <c r="F14" s="17" t="s">
         <v>24</v>
@@ -3213,46 +3193,46 @@
       <c r="J14" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="K14" s="69" t="s">
-        <v>74</v>
+      <c r="K14" s="38" t="s">
+        <v>72</v>
       </c>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
     </row>
     <row r="15" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
-      <c r="B15" s="68"/>
-      <c r="C15" s="68"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="37"/>
       <c r="D15" s="7"/>
-      <c r="E15" s="68"/>
-      <c r="F15" s="68"/>
-      <c r="G15" s="68"/>
-      <c r="H15" s="68"/>
-      <c r="I15" s="68"/>
-      <c r="J15" s="68"/>
-      <c r="K15" s="68"/>
-      <c r="L15" s="68"/>
-      <c r="M15" s="68"/>
-      <c r="N15" s="68"/>
+      <c r="E15" s="37"/>
+      <c r="F15" s="37"/>
+      <c r="G15" s="37"/>
+      <c r="H15" s="37"/>
+      <c r="I15" s="37"/>
+      <c r="J15" s="37"/>
+      <c r="K15" s="37"/>
+      <c r="L15" s="37"/>
+      <c r="M15" s="37"/>
+      <c r="N15" s="37"/>
       <c r="O15" s="1"/>
       <c r="P15" s="1"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="68" t="s">
-        <v>79</v>
-      </c>
-      <c r="C16" s="68"/>
+      <c r="B16" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16" s="37"/>
       <c r="D16" s="7"/>
-      <c r="E16" s="68"/>
-      <c r="F16" s="71"/>
-      <c r="G16" s="71"/>
-      <c r="H16" s="71"/>
-      <c r="I16" s="71"/>
-      <c r="J16" s="71"/>
-      <c r="K16" s="86"/>
-      <c r="L16" s="86"/>
-      <c r="M16" s="71"/>
+      <c r="E16" s="37"/>
+      <c r="F16" s="40"/>
+      <c r="G16" s="40"/>
+      <c r="H16" s="40"/>
+      <c r="I16" s="40"/>
+      <c r="J16" s="40"/>
+      <c r="K16" s="100"/>
+      <c r="L16" s="100"/>
+      <c r="M16" s="40"/>
       <c r="N16" s="1"/>
       <c r="O16" s="1"/>
       <c r="P16" s="1"/>
@@ -3270,7 +3250,7 @@
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
-      <c r="M17" s="71"/>
+      <c r="M17" s="40"/>
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
       <c r="P17" s="1"/>
@@ -3278,132 +3258,132 @@
     <row r="18" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
-      <c r="C18" s="87" t="s">
+      <c r="C18" s="101" t="s">
+        <v>78</v>
+      </c>
+      <c r="D18" s="102"/>
+      <c r="E18" s="102"/>
+      <c r="F18" s="103"/>
+      <c r="G18" s="41" t="s">
+        <v>79</v>
+      </c>
+      <c r="H18" s="101" t="s">
         <v>80</v>
       </c>
-      <c r="D18" s="88"/>
-      <c r="E18" s="88"/>
-      <c r="F18" s="89"/>
-      <c r="G18" s="72" t="s">
+      <c r="I18" s="102"/>
+      <c r="J18" s="102"/>
+      <c r="K18" s="102"/>
+      <c r="L18" s="103"/>
+      <c r="M18" s="101" t="s">
         <v>81</v>
       </c>
-      <c r="H18" s="87" t="s">
-        <v>82</v>
-      </c>
-      <c r="I18" s="88"/>
-      <c r="J18" s="88"/>
-      <c r="K18" s="88"/>
-      <c r="L18" s="89"/>
-      <c r="M18" s="87" t="s">
-        <v>83</v>
-      </c>
-      <c r="N18" s="88"/>
-      <c r="O18" s="88"/>
-      <c r="P18" s="90"/>
+      <c r="N18" s="102"/>
+      <c r="O18" s="102"/>
+      <c r="P18" s="104"/>
     </row>
     <row r="19" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
-      <c r="B19" s="80" t="s">
-        <v>67</v>
-      </c>
-      <c r="C19" s="92" t="s">
+      <c r="B19" s="85" t="s">
+        <v>66</v>
+      </c>
+      <c r="C19" s="91" t="s">
+        <v>82</v>
+      </c>
+      <c r="D19" s="67" t="s">
+        <v>83</v>
+      </c>
+      <c r="E19" s="67" t="s">
         <v>84</v>
       </c>
-      <c r="D19" s="33" t="s">
+      <c r="F19" s="85" t="s">
         <v>85</v>
       </c>
-      <c r="E19" s="33" t="s">
+      <c r="G19" s="105" t="s">
         <v>86</v>
       </c>
-      <c r="F19" s="80" t="s">
+      <c r="H19" s="95" t="s">
         <v>87</v>
       </c>
-      <c r="G19" s="94" t="s">
-        <v>88</v>
-      </c>
-      <c r="H19" s="96" t="s">
-        <v>89</v>
-      </c>
-      <c r="I19" s="97"/>
-      <c r="J19" s="33" t="s">
+      <c r="I19" s="96"/>
+      <c r="J19" s="67" t="s">
+        <v>82</v>
+      </c>
+      <c r="K19" s="67" t="s">
+        <v>83</v>
+      </c>
+      <c r="L19" s="85" t="s">
         <v>84</v>
       </c>
-      <c r="K19" s="33" t="s">
-        <v>85</v>
-      </c>
-      <c r="L19" s="80" t="s">
-        <v>86</v>
-      </c>
-      <c r="M19" s="82" t="s">
-        <v>89</v>
-      </c>
-      <c r="N19" s="33" t="s">
+      <c r="M19" s="87" t="s">
+        <v>87</v>
+      </c>
+      <c r="N19" s="67" t="s">
+        <v>82</v>
+      </c>
+      <c r="O19" s="67" t="s">
+        <v>83</v>
+      </c>
+      <c r="P19" s="85" t="s">
         <v>84</v>
-      </c>
-      <c r="O19" s="33" t="s">
-        <v>85</v>
-      </c>
-      <c r="P19" s="80" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
-      <c r="B20" s="91"/>
-      <c r="C20" s="93"/>
-      <c r="D20" s="34"/>
-      <c r="E20" s="34"/>
-      <c r="F20" s="91"/>
-      <c r="G20" s="95"/>
-      <c r="H20" s="98"/>
-      <c r="I20" s="99"/>
-      <c r="J20" s="34"/>
-      <c r="K20" s="34"/>
-      <c r="L20" s="91"/>
-      <c r="M20" s="100"/>
-      <c r="N20" s="34"/>
-      <c r="O20" s="34"/>
-      <c r="P20" s="91"/>
+      <c r="B20" s="90"/>
+      <c r="C20" s="92"/>
+      <c r="D20" s="68"/>
+      <c r="E20" s="68"/>
+      <c r="F20" s="90"/>
+      <c r="G20" s="106"/>
+      <c r="H20" s="97"/>
+      <c r="I20" s="98"/>
+      <c r="J20" s="68"/>
+      <c r="K20" s="68"/>
+      <c r="L20" s="90"/>
+      <c r="M20" s="99"/>
+      <c r="N20" s="68"/>
+      <c r="O20" s="68"/>
+      <c r="P20" s="90"/>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
-      <c r="B21" s="73" t="s">
-        <v>71</v>
-      </c>
-      <c r="C21" s="74">
+      <c r="B21" s="42" t="s">
+        <v>70</v>
+      </c>
+      <c r="C21" s="43">
         <v>8</v>
       </c>
-      <c r="D21" s="75">
+      <c r="D21" s="44">
         <v>5</v>
       </c>
-      <c r="E21" s="75">
+      <c r="E21" s="44">
         <v>3</v>
       </c>
-      <c r="F21" s="76"/>
-      <c r="G21" s="77"/>
-      <c r="H21" s="101" t="s">
-        <v>90</v>
-      </c>
-      <c r="I21" s="102"/>
+      <c r="F21" s="45"/>
+      <c r="G21" s="46"/>
+      <c r="H21" s="93" t="s">
+        <v>88</v>
+      </c>
+      <c r="I21" s="94"/>
       <c r="J21" s="4">
         <v>3</v>
       </c>
-      <c r="K21" s="75">
+      <c r="K21" s="44">
         <v>3</v>
       </c>
-      <c r="L21" s="76">
+      <c r="L21" s="45">
         <v>0</v>
       </c>
-      <c r="M21" s="78" t="s">
-        <v>90</v>
+      <c r="M21" s="47" t="s">
+        <v>88</v>
       </c>
       <c r="N21" s="4">
         <v>5</v>
       </c>
-      <c r="O21" s="75">
+      <c r="O21" s="44">
         <v>5</v>
       </c>
-      <c r="P21" s="76">
+      <c r="P21" s="45">
         <v>0</v>
       </c>
     </row>
@@ -3420,7 +3400,7 @@
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
       <c r="L22" s="1"/>
-      <c r="M22" s="51"/>
+      <c r="M22" s="25"/>
       <c r="N22" s="1"/>
       <c r="O22" s="1"/>
       <c r="P22" s="1"/>
@@ -3441,19 +3421,19 @@
     <mergeCell ref="C18:F18"/>
     <mergeCell ref="H18:L18"/>
     <mergeCell ref="M18:P18"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="C6:C14"/>
     <mergeCell ref="B19:B20"/>
     <mergeCell ref="C19:C20"/>
     <mergeCell ref="D19:D20"/>
     <mergeCell ref="E19:E20"/>
     <mergeCell ref="F19:F20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="C6:C14"/>
+    <mergeCell ref="J4:K4"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="C4:C5"/>
     <mergeCell ref="D4:D5"/>
     <mergeCell ref="E4:E5"/>
-    <mergeCell ref="J4:K4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>